<commit_message>
Publish catalog from admin
</commit_message>
<xml_diff>
--- a/data/Euro_Coin_Catalog_Automation.xlsx
+++ b/data/Euro_Coin_Catalog_Automation.xlsx
@@ -9001,80 +9001,316 @@
       </c>
     </row>
     <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="5" t="n"/>
-      <c r="B115" s="6" t="n"/>
-      <c r="C115" s="5" t="n"/>
-      <c r="D115" s="7" t="n"/>
-      <c r="E115" s="6" t="n"/>
-      <c r="F115" s="6" t="n"/>
-      <c r="G115" s="6" t="n"/>
-      <c r="H115" s="6" t="n"/>
-      <c r="I115" s="6" t="n"/>
-      <c r="J115" s="7" t="n"/>
-      <c r="K115" s="5" t="n"/>
-      <c r="L115" s="6" t="n"/>
-      <c r="M115" s="5" t="n"/>
-      <c r="N115" s="5" t="n"/>
-      <c r="O115" s="5" t="n"/>
-      <c r="P115" s="8" t="n"/>
-      <c r="Q115" s="9" t="n"/>
+      <c r="A115" s="12" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E115" s="13" t="inlineStr">
+        <is>
+          <t>1 cent</t>
+        </is>
+      </c>
+      <c r="F115" s="13" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="G115" s="13" t="inlineStr">
+        <is>
+          <t>1 cent</t>
+        </is>
+      </c>
+      <c r="H115" s="13" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I115" s="13" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J115" s="14" t="inlineStr"/>
+      <c r="K115" s="12" t="inlineStr">
+        <is>
+          <t>116_Austria_2013_1cent_Regular.jpeg</t>
+        </is>
+      </c>
+      <c r="L115" s="13" t="inlineStr"/>
+      <c r="M115" s="12" t="inlineStr">
+        <is>
+          <t>Copper-plated steel</t>
+        </is>
+      </c>
+      <c r="N115" s="12" t="inlineStr">
+        <is>
+          <t>2.30 g</t>
+        </is>
+      </c>
+      <c r="O115" s="12" t="inlineStr">
+        <is>
+          <t>16.25 mm</t>
+        </is>
+      </c>
+      <c r="P115" s="15" t="inlineStr">
+        <is>
+          <t>Regular 1 cent circulation coin of Austria.</t>
+        </is>
+      </c>
+      <c r="Q115" s="16" t="inlineStr">
+        <is>
+          <t>Austria chose to produce a series of coins illustrating flowers, architecture and famous people from its history. The designs were chosen by a national panel and public opinion poll. Austrian artist Josef Kaiser created the designs.
+This coin features a gentian, as part of a floral series, symbolising a duty to the environment and the part Austria is playing in the development of a Community environmental policy.</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1">
-      <c r="A116" s="5" t="n"/>
-      <c r="B116" s="6" t="n"/>
-      <c r="C116" s="5" t="n"/>
-      <c r="D116" s="7" t="n"/>
-      <c r="E116" s="6" t="n"/>
-      <c r="F116" s="6" t="n"/>
-      <c r="G116" s="6" t="n"/>
-      <c r="H116" s="6" t="n"/>
-      <c r="I116" s="6" t="n"/>
-      <c r="J116" s="7" t="n"/>
-      <c r="K116" s="5" t="n"/>
-      <c r="L116" s="6" t="n"/>
-      <c r="M116" s="5" t="n"/>
-      <c r="N116" s="5" t="n"/>
-      <c r="O116" s="5" t="n"/>
-      <c r="P116" s="8" t="n"/>
-      <c r="Q116" s="9" t="n"/>
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E116" s="13" t="inlineStr">
+        <is>
+          <t>2 cent</t>
+        </is>
+      </c>
+      <c r="F116" s="13" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="G116" s="13" t="inlineStr">
+        <is>
+          <t>2 cent</t>
+        </is>
+      </c>
+      <c r="H116" s="13" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I116" s="13" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J116" s="14" t="inlineStr"/>
+      <c r="K116" s="12" t="inlineStr">
+        <is>
+          <t>117_Austria_2013_2cent_Regular.jpeg</t>
+        </is>
+      </c>
+      <c r="L116" s="13" t="inlineStr"/>
+      <c r="M116" s="12" t="inlineStr">
+        <is>
+          <t>Copper-plated steel</t>
+        </is>
+      </c>
+      <c r="N116" s="12" t="inlineStr">
+        <is>
+          <t>3.06 g</t>
+        </is>
+      </c>
+      <c r="O116" s="12" t="inlineStr">
+        <is>
+          <t>18.75 mm</t>
+        </is>
+      </c>
+      <c r="P116" s="15" t="inlineStr">
+        <is>
+          <t>Regular 2 cent circulation coin of Austria.</t>
+        </is>
+      </c>
+      <c r="Q116" s="16" t="inlineStr">
+        <is>
+          <t>Austria chose to produce a series of coins illustrating flowers, architecture and famous people from its history. The designs were chosen by a national panel and public opinion poll. Austrian artist Josef Kaiser created the designs.
+This coin features an edelweiss, as part of a floral series, symbolising a duty to the environment and the part Austria is playing in the development of a Community environmental policy.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="5" t="n"/>
-      <c r="B117" s="6" t="n"/>
-      <c r="C117" s="5" t="n"/>
-      <c r="D117" s="7" t="n"/>
-      <c r="E117" s="6" t="n"/>
-      <c r="F117" s="6" t="n"/>
-      <c r="G117" s="6" t="n"/>
-      <c r="H117" s="6" t="n"/>
-      <c r="I117" s="6" t="n"/>
-      <c r="J117" s="7" t="n"/>
-      <c r="K117" s="5" t="n"/>
-      <c r="L117" s="6" t="n"/>
-      <c r="M117" s="5" t="n"/>
-      <c r="N117" s="5" t="n"/>
-      <c r="O117" s="5" t="n"/>
-      <c r="P117" s="8" t="n"/>
-      <c r="Q117" s="9" t="n"/>
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D117" s="14" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E117" s="13" t="inlineStr">
+        <is>
+          <t>5 cent</t>
+        </is>
+      </c>
+      <c r="F117" s="13" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="G117" s="13" t="inlineStr">
+        <is>
+          <t>5 cent</t>
+        </is>
+      </c>
+      <c r="H117" s="13" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I117" s="13" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J117" s="14" t="inlineStr"/>
+      <c r="K117" s="12" t="inlineStr">
+        <is>
+          <t>118_Austria_2002_5cent_Regular.jpeg</t>
+        </is>
+      </c>
+      <c r="L117" s="13" t="inlineStr"/>
+      <c r="M117" s="12" t="inlineStr">
+        <is>
+          <t>Copper-plated steel</t>
+        </is>
+      </c>
+      <c r="N117" s="12" t="inlineStr">
+        <is>
+          <t>3.92 g</t>
+        </is>
+      </c>
+      <c r="O117" s="12" t="inlineStr">
+        <is>
+          <t>21.25 mm</t>
+        </is>
+      </c>
+      <c r="P117" s="15" t="inlineStr">
+        <is>
+          <t>Regular 5 cent circulation coin of Austria.</t>
+        </is>
+      </c>
+      <c r="Q117" s="16" t="inlineStr">
+        <is>
+          <t>Austria chose to produce a series of coins illustrating flowers, architecture and famous people from its history. The designs were chosen by a national panel and public opinion poll. Austrian artist Josef Kaiser created the designs.
+This coin features alpine primroses, as part of a floral series, symbolising a duty to the environment and the part Austria is playing in the development of a Community environmental policy.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1">
-      <c r="A118" s="5" t="n"/>
-      <c r="B118" s="6" t="n"/>
-      <c r="C118" s="5" t="n"/>
-      <c r="D118" s="7" t="n"/>
-      <c r="E118" s="6" t="n"/>
-      <c r="F118" s="6" t="n"/>
-      <c r="G118" s="6" t="n"/>
-      <c r="H118" s="6" t="n"/>
-      <c r="I118" s="6" t="n"/>
-      <c r="J118" s="7" t="n"/>
-      <c r="K118" s="5" t="n"/>
-      <c r="L118" s="6" t="n"/>
-      <c r="M118" s="5" t="n"/>
-      <c r="N118" s="5" t="n"/>
-      <c r="O118" s="5" t="n"/>
-      <c r="P118" s="8" t="n"/>
-      <c r="Q118" s="9" t="n"/>
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B118" s="13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E118" s="13" t="inlineStr">
+        <is>
+          <t>10 cent</t>
+        </is>
+      </c>
+      <c r="F118" s="13" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="G118" s="13" t="inlineStr">
+        <is>
+          <t>10 cent</t>
+        </is>
+      </c>
+      <c r="H118" s="13" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I118" s="13" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J118" s="14" t="inlineStr"/>
+      <c r="K118" s="12" t="inlineStr">
+        <is>
+          <t>119_Austria_2011_10cent_Regular.jpeg</t>
+        </is>
+      </c>
+      <c r="L118" s="13" t="inlineStr"/>
+      <c r="M118" s="12" t="inlineStr">
+        <is>
+          <t>Nordic gold</t>
+        </is>
+      </c>
+      <c r="N118" s="12" t="inlineStr">
+        <is>
+          <t>4.10 g</t>
+        </is>
+      </c>
+      <c r="O118" s="12" t="inlineStr">
+        <is>
+          <t>19.75 mm</t>
+        </is>
+      </c>
+      <c r="P118" s="15" t="inlineStr">
+        <is>
+          <t>Regular 10 cent circulation coin of Austria.</t>
+        </is>
+      </c>
+      <c r="Q118" s="16" t="inlineStr">
+        <is>
+          <t>Austria chose to produce a series of coins illustrating flowers, architecture and famous people from its history. The designs were chosen by a national panel and public opinion poll. Austrian artist Josef Kaiser created the designs.
+St. Stephen's Cathedral, one of the jewels of Viennese Gothic architecture and a popular tourist venue, is depicted on this coin.</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1">
       <c r="A119" s="5" t="n"/>

</xml_diff>